<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-14 (sentiment: 35.27)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J479"/>
+  <dimension ref="A1:J480"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15762,7 +15762,7 @@
         <v>58.5</v>
       </c>
       <c r="E479" t="n">
-        <v>5.58</v>
+        <v>6.54</v>
       </c>
       <c r="F479" t="n">
         <v>5.16</v>
@@ -15778,6 +15778,38 @@
       </c>
       <c r="J479" t="n">
         <v>32.19</v>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" s="2" t="n">
+        <v>46279.66666666666</v>
+      </c>
+      <c r="B480" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C480" t="n">
+        <v>42.28</v>
+      </c>
+      <c r="D480" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E480" t="n">
+        <v>7.84</v>
+      </c>
+      <c r="F480" t="n">
+        <v>5.36</v>
+      </c>
+      <c r="G480" t="n">
+        <v>66.47</v>
+      </c>
+      <c r="H480" t="n">
+        <v>64.68000000000001</v>
+      </c>
+      <c r="I480" t="n">
+        <v>4.56</v>
+      </c>
+      <c r="J480" t="n">
+        <v>35.27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-15 (sentiment: 34.47)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J480"/>
+  <dimension ref="A1:J481"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15794,7 +15794,7 @@
         <v>58.5</v>
       </c>
       <c r="E480" t="n">
-        <v>7.84</v>
+        <v>6.44</v>
       </c>
       <c r="F480" t="n">
         <v>5.36</v>
@@ -15806,10 +15806,42 @@
         <v>64.68000000000001</v>
       </c>
       <c r="I480" t="n">
-        <v>4.56</v>
+        <v>0.2</v>
       </c>
       <c r="J480" t="n">
-        <v>35.27</v>
+        <v>34.18</v>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" s="2" t="n">
+        <v>46280.66666666666</v>
+      </c>
+      <c r="B481" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C481" t="n">
+        <v>42.45</v>
+      </c>
+      <c r="D481" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E481" t="n">
+        <v>6.52</v>
+      </c>
+      <c r="F481" t="n">
+        <v>5.56</v>
+      </c>
+      <c r="G481" t="n">
+        <v>66.87</v>
+      </c>
+      <c r="H481" t="n">
+        <v>64.88</v>
+      </c>
+      <c r="I481" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="J481" t="n">
+        <v>34.47</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-16 (sentiment: 34.87)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J481"/>
+  <dimension ref="A1:J482"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15826,7 +15826,7 @@
         <v>58.5</v>
       </c>
       <c r="E481" t="n">
-        <v>6.52</v>
+        <v>6.71</v>
       </c>
       <c r="F481" t="n">
         <v>5.56</v>
@@ -15838,10 +15838,42 @@
         <v>64.88</v>
       </c>
       <c r="I481" t="n">
-        <v>0.6</v>
+        <v>2.18</v>
       </c>
       <c r="J481" t="n">
-        <v>34.47</v>
+        <v>34.87</v>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" s="2" t="n">
+        <v>46281.66666666666</v>
+      </c>
+      <c r="B482" t="n">
+        <v>1.48</v>
+      </c>
+      <c r="C482" t="n">
+        <v>43.01</v>
+      </c>
+      <c r="D482" t="n">
+        <v>58.5</v>
+      </c>
+      <c r="E482" t="n">
+        <v>5.83</v>
+      </c>
+      <c r="F482" t="n">
+        <v>5.75</v>
+      </c>
+      <c r="G482" t="n">
+        <v>68.84999999999999</v>
+      </c>
+      <c r="H482" t="n">
+        <v>64.68000000000001</v>
+      </c>
+      <c r="I482" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J482" t="n">
+        <v>34.87</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-16 (sentiment: 23.54)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -15371,9 +15371,7 @@
       <c r="B467" t="n">
         <v>1.48</v>
       </c>
-      <c r="C467" t="n">
-        <v>43.5</v>
-      </c>
+      <c r="C467" t="inlineStr"/>
       <c r="D467" t="n">
         <v>58.5</v>
       </c>
@@ -15383,9 +15381,7 @@
       <c r="F467" t="n">
         <v>2.78</v>
       </c>
-      <c r="G467" t="n">
-        <v>71.23</v>
-      </c>
+      <c r="G467" t="inlineStr"/>
       <c r="H467" t="n">
         <v>65.67</v>
       </c>
@@ -15393,7 +15389,7 @@
         <v>5.75</v>
       </c>
       <c r="J467" t="n">
-        <v>36.36</v>
+        <v>24.74</v>
       </c>
     </row>
     <row r="468">
@@ -15403,9 +15399,7 @@
       <c r="B468" t="n">
         <v>1.48</v>
       </c>
-      <c r="C468" t="n">
-        <v>42.15</v>
-      </c>
+      <c r="C468" t="inlineStr"/>
       <c r="D468" t="n">
         <v>58.5</v>
       </c>
@@ -15415,9 +15409,7 @@
       <c r="F468" t="n">
         <v>2.98</v>
       </c>
-      <c r="G468" t="n">
-        <v>66.87</v>
-      </c>
+      <c r="G468" t="inlineStr"/>
       <c r="H468" t="n">
         <v>65.48</v>
       </c>
@@ -15425,7 +15417,7 @@
         <v>35.91</v>
       </c>
       <c r="J468" t="n">
-        <v>42.81</v>
+        <v>34.79</v>
       </c>
     </row>
     <row r="469">
@@ -15435,9 +15427,7 @@
       <c r="B469" t="n">
         <v>1.48</v>
       </c>
-      <c r="C469" t="n">
-        <v>42.15</v>
-      </c>
+      <c r="C469" t="inlineStr"/>
       <c r="D469" t="n">
         <v>58.5</v>
       </c>
@@ -15447,9 +15437,7 @@
       <c r="F469" t="n">
         <v>3.17</v>
       </c>
-      <c r="G469" t="n">
-        <v>66.67</v>
-      </c>
+      <c r="G469" t="inlineStr"/>
       <c r="H469" t="n">
         <v>65.28</v>
       </c>
@@ -15457,7 +15445,7 @@
         <v>12.9</v>
       </c>
       <c r="J469" t="n">
-        <v>37</v>
+        <v>27.12</v>
       </c>
     </row>
     <row r="470">
@@ -15467,9 +15455,7 @@
       <c r="B470" t="n">
         <v>1.48</v>
       </c>
-      <c r="C470" t="n">
-        <v>42.9</v>
-      </c>
+      <c r="C470" t="inlineStr"/>
       <c r="D470" t="n">
         <v>58.5</v>
       </c>
@@ -15479,9 +15465,7 @@
       <c r="F470" t="n">
         <v>3.37</v>
       </c>
-      <c r="G470" t="n">
-        <v>68.84999999999999</v>
-      </c>
+      <c r="G470" t="inlineStr"/>
       <c r="H470" t="n">
         <v>65.48</v>
       </c>
@@ -15489,7 +15473,7 @@
         <v>0.2</v>
       </c>
       <c r="J470" t="n">
-        <v>34.47</v>
+        <v>23.02</v>
       </c>
     </row>
     <row r="471">
@@ -15499,9 +15483,7 @@
       <c r="B471" t="n">
         <v>1.48</v>
       </c>
-      <c r="C471" t="n">
-        <v>41.75</v>
-      </c>
+      <c r="C471" t="inlineStr"/>
       <c r="D471" t="n">
         <v>58.5</v>
       </c>
@@ -15511,9 +15493,7 @@
       <c r="F471" t="n">
         <v>3.57</v>
       </c>
-      <c r="G471" t="n">
-        <v>64.48</v>
-      </c>
+      <c r="G471" t="inlineStr"/>
       <c r="H471" t="n">
         <v>65.67</v>
       </c>
@@ -15521,7 +15501,7 @@
         <v>0.2</v>
       </c>
       <c r="J471" t="n">
-        <v>33.48</v>
+        <v>23.15</v>
       </c>
     </row>
     <row r="472">
@@ -15531,9 +15511,7 @@
       <c r="B472" t="n">
         <v>1.48</v>
       </c>
-      <c r="C472" t="n">
-        <v>40.51</v>
-      </c>
+      <c r="C472" t="inlineStr"/>
       <c r="D472" t="n">
         <v>58.5</v>
       </c>
@@ -15543,9 +15521,7 @@
       <c r="F472" t="n">
         <v>3.77</v>
       </c>
-      <c r="G472" t="n">
-        <v>58.93</v>
-      </c>
+      <c r="G472" t="inlineStr"/>
       <c r="H472" t="n">
         <v>65.48</v>
       </c>
@@ -15553,7 +15529,7 @@
         <v>0.2</v>
       </c>
       <c r="J472" t="n">
-        <v>32.09</v>
+        <v>23.15</v>
       </c>
     </row>
     <row r="473">
@@ -15563,9 +15539,7 @@
       <c r="B473" t="n">
         <v>1.48</v>
       </c>
-      <c r="C473" t="n">
-        <v>41.73</v>
-      </c>
+      <c r="C473" t="inlineStr"/>
       <c r="D473" t="n">
         <v>58.5</v>
       </c>
@@ -15575,9 +15549,7 @@
       <c r="F473" t="n">
         <v>3.97</v>
       </c>
-      <c r="G473" t="n">
-        <v>64.09</v>
-      </c>
+      <c r="G473" t="inlineStr"/>
       <c r="H473" t="n">
         <v>65.67</v>
       </c>
@@ -15585,7 +15557,7 @@
         <v>0.6</v>
       </c>
       <c r="J473" t="n">
-        <v>33.58</v>
+        <v>23.41</v>
       </c>
     </row>
     <row r="474">
@@ -15595,9 +15567,7 @@
       <c r="B474" t="n">
         <v>1.48</v>
       </c>
-      <c r="C474" t="n">
-        <v>41.57</v>
-      </c>
+      <c r="C474" t="inlineStr"/>
       <c r="D474" t="n">
         <v>58.5</v>
       </c>
@@ -15607,9 +15577,7 @@
       <c r="F474" t="n">
         <v>4.17</v>
       </c>
-      <c r="G474" t="n">
-        <v>63.29</v>
-      </c>
+      <c r="G474" t="inlineStr"/>
       <c r="H474" t="n">
         <v>65.48</v>
       </c>
@@ -15617,7 +15585,7 @@
         <v>0.2</v>
       </c>
       <c r="J474" t="n">
-        <v>33.28</v>
+        <v>23.28</v>
       </c>
     </row>
     <row r="475">
@@ -15627,9 +15595,7 @@
       <c r="B475" t="n">
         <v>1.48</v>
       </c>
-      <c r="C475" t="n">
-        <v>42.75</v>
-      </c>
+      <c r="C475" t="inlineStr"/>
       <c r="D475" t="n">
         <v>58.5</v>
       </c>
@@ -15639,9 +15605,7 @@
       <c r="F475" t="n">
         <v>4.37</v>
       </c>
-      <c r="G475" t="n">
-        <v>68.06</v>
-      </c>
+      <c r="G475" t="inlineStr"/>
       <c r="H475" t="n">
         <v>65.28</v>
       </c>
@@ -15649,7 +15613,7 @@
         <v>1.79</v>
       </c>
       <c r="J475" t="n">
-        <v>34.87</v>
+        <v>23.81</v>
       </c>
     </row>
     <row r="476">
@@ -15659,9 +15623,7 @@
       <c r="B476" t="n">
         <v>1.48</v>
       </c>
-      <c r="C476" t="n">
-        <v>41.65</v>
-      </c>
+      <c r="C476" t="inlineStr"/>
       <c r="D476" t="n">
         <v>58.5</v>
       </c>
@@ -15671,9 +15633,7 @@
       <c r="F476" t="n">
         <v>4.56</v>
       </c>
-      <c r="G476" t="n">
-        <v>63.29</v>
-      </c>
+      <c r="G476" t="inlineStr"/>
       <c r="H476" t="n">
         <v>65.48</v>
       </c>
@@ -15681,7 +15641,7 @@
         <v>1.79</v>
       </c>
       <c r="J476" t="n">
-        <v>33.78</v>
+        <v>23.94</v>
       </c>
     </row>
     <row r="477">
@@ -15691,9 +15651,7 @@
       <c r="B477" t="n">
         <v>1.48</v>
       </c>
-      <c r="C477" t="n">
-        <v>40.6</v>
-      </c>
+      <c r="C477" t="inlineStr"/>
       <c r="D477" t="n">
         <v>58.5</v>
       </c>
@@ -15703,9 +15661,7 @@
       <c r="F477" t="n">
         <v>4.76</v>
       </c>
-      <c r="G477" t="n">
-        <v>57.74</v>
-      </c>
+      <c r="G477" t="inlineStr"/>
       <c r="H477" t="n">
         <v>65.28</v>
       </c>
@@ -15713,7 +15669,7 @@
         <v>0.99</v>
       </c>
       <c r="J477" t="n">
-        <v>32.19</v>
+        <v>23.68</v>
       </c>
     </row>
     <row r="478">
@@ -15723,9 +15679,7 @@
       <c r="B478" t="n">
         <v>1.48</v>
       </c>
-      <c r="C478" t="n">
-        <v>40.73</v>
-      </c>
+      <c r="C478" t="inlineStr"/>
       <c r="D478" t="n">
         <v>58.5</v>
       </c>
@@ -15735,9 +15689,7 @@
       <c r="F478" t="n">
         <v>4.96</v>
       </c>
-      <c r="G478" t="n">
-        <v>58.13</v>
-      </c>
+      <c r="G478" t="inlineStr"/>
       <c r="H478" t="n">
         <v>65.08</v>
       </c>
@@ -15745,7 +15697,7 @@
         <v>0.99</v>
       </c>
       <c r="J478" t="n">
-        <v>32.29</v>
+        <v>23.68</v>
       </c>
     </row>
     <row r="479">
@@ -15755,9 +15707,7 @@
       <c r="B479" t="n">
         <v>1.48</v>
       </c>
-      <c r="C479" t="n">
-        <v>40.81</v>
-      </c>
+      <c r="C479" t="inlineStr"/>
       <c r="D479" t="n">
         <v>58.5</v>
       </c>
@@ -15767,9 +15717,7 @@
       <c r="F479" t="n">
         <v>5.16</v>
       </c>
-      <c r="G479" t="n">
-        <v>58.53</v>
-      </c>
+      <c r="G479" t="inlineStr"/>
       <c r="H479" t="n">
         <v>64.88</v>
       </c>
@@ -15777,7 +15725,7 @@
         <v>0.2</v>
       </c>
       <c r="J479" t="n">
-        <v>32.19</v>
+        <v>23.41</v>
       </c>
     </row>
     <row r="480">
@@ -15787,9 +15735,7 @@
       <c r="B480" t="n">
         <v>1.48</v>
       </c>
-      <c r="C480" t="n">
-        <v>42.28</v>
-      </c>
+      <c r="C480" t="inlineStr"/>
       <c r="D480" t="n">
         <v>58.5</v>
       </c>
@@ -15799,9 +15745,7 @@
       <c r="F480" t="n">
         <v>5.36</v>
       </c>
-      <c r="G480" t="n">
-        <v>66.47</v>
-      </c>
+      <c r="G480" t="inlineStr"/>
       <c r="H480" t="n">
         <v>64.68000000000001</v>
       </c>
@@ -15809,7 +15753,7 @@
         <v>0.2</v>
       </c>
       <c r="J480" t="n">
-        <v>34.18</v>
+        <v>23.41</v>
       </c>
     </row>
     <row r="481">
@@ -15819,9 +15763,7 @@
       <c r="B481" t="n">
         <v>1.48</v>
       </c>
-      <c r="C481" t="n">
-        <v>42.45</v>
-      </c>
+      <c r="C481" t="inlineStr"/>
       <c r="D481" t="n">
         <v>58.5</v>
       </c>
@@ -15831,9 +15773,7 @@
       <c r="F481" t="n">
         <v>5.56</v>
       </c>
-      <c r="G481" t="n">
-        <v>66.87</v>
-      </c>
+      <c r="G481" t="inlineStr"/>
       <c r="H481" t="n">
         <v>64.88</v>
       </c>
@@ -15841,7 +15781,7 @@
         <v>2.18</v>
       </c>
       <c r="J481" t="n">
-        <v>34.87</v>
+        <v>24.21</v>
       </c>
     </row>
     <row r="482">
@@ -15851,9 +15791,7 @@
       <c r="B482" t="n">
         <v>1.48</v>
       </c>
-      <c r="C482" t="n">
-        <v>43.01</v>
-      </c>
+      <c r="C482" t="inlineStr"/>
       <c r="D482" t="n">
         <v>58.5</v>
       </c>
@@ -15863,9 +15801,7 @@
       <c r="F482" t="n">
         <v>5.75</v>
       </c>
-      <c r="G482" t="n">
-        <v>68.84999999999999</v>
-      </c>
+      <c r="G482" t="inlineStr"/>
       <c r="H482" t="n">
         <v>64.68000000000001</v>
       </c>
@@ -15873,7 +15809,7 @@
         <v>0.2</v>
       </c>
       <c r="J482" t="n">
-        <v>34.87</v>
+        <v>23.54</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-16 (sentiment: 38.99)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -15651,7 +15651,9 @@
       <c r="B477" t="n">
         <v>1.48</v>
       </c>
-      <c r="C477" t="inlineStr"/>
+      <c r="C477" t="n">
+        <v>39.19</v>
+      </c>
       <c r="D477" t="n">
         <v>58.5</v>
       </c>
@@ -15661,7 +15663,9 @@
       <c r="F477" t="n">
         <v>4.76</v>
       </c>
-      <c r="G477" t="inlineStr"/>
+      <c r="G477" t="n">
+        <v>53.51</v>
+      </c>
       <c r="H477" t="n">
         <v>65.28</v>
       </c>
@@ -15669,7 +15673,7 @@
         <v>0.99</v>
       </c>
       <c r="J477" t="n">
-        <v>23.68</v>
+        <v>31.14</v>
       </c>
     </row>
     <row r="478">
@@ -15679,7 +15683,9 @@
       <c r="B478" t="n">
         <v>1.48</v>
       </c>
-      <c r="C478" t="inlineStr"/>
+      <c r="C478" t="n">
+        <v>38.33</v>
+      </c>
       <c r="D478" t="n">
         <v>58.5</v>
       </c>
@@ -15689,7 +15695,9 @@
       <c r="F478" t="n">
         <v>4.96</v>
       </c>
-      <c r="G478" t="inlineStr"/>
+      <c r="G478" t="n">
+        <v>47.73</v>
+      </c>
       <c r="H478" t="n">
         <v>65.08</v>
       </c>
@@ -15697,7 +15705,7 @@
         <v>0.99</v>
       </c>
       <c r="J478" t="n">
-        <v>23.68</v>
+        <v>29.69</v>
       </c>
     </row>
     <row r="479">
@@ -15707,7 +15715,9 @@
       <c r="B479" t="n">
         <v>1.48</v>
       </c>
-      <c r="C479" t="inlineStr"/>
+      <c r="C479" t="n">
+        <v>41.04</v>
+      </c>
       <c r="D479" t="n">
         <v>58.5</v>
       </c>
@@ -15717,7 +15727,9 @@
       <c r="F479" t="n">
         <v>5.16</v>
       </c>
-      <c r="G479" t="inlineStr"/>
+      <c r="G479" t="n">
+        <v>61.78</v>
+      </c>
       <c r="H479" t="n">
         <v>64.88</v>
       </c>
@@ -15725,7 +15737,7 @@
         <v>0.2</v>
       </c>
       <c r="J479" t="n">
-        <v>23.41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="480">
@@ -15735,7 +15747,9 @@
       <c r="B480" t="n">
         <v>1.48</v>
       </c>
-      <c r="C480" t="inlineStr"/>
+      <c r="C480" t="n">
+        <v>42.14</v>
+      </c>
       <c r="D480" t="n">
         <v>58.5</v>
       </c>
@@ -15745,7 +15759,9 @@
       <c r="F480" t="n">
         <v>5.36</v>
       </c>
-      <c r="G480" t="inlineStr"/>
+      <c r="G480" t="n">
+        <v>65.91</v>
+      </c>
       <c r="H480" t="n">
         <v>64.68000000000001</v>
       </c>
@@ -15753,7 +15769,7 @@
         <v>0.2</v>
       </c>
       <c r="J480" t="n">
-        <v>23.41</v>
+        <v>34.04</v>
       </c>
     </row>
     <row r="481">
@@ -15763,7 +15779,9 @@
       <c r="B481" t="n">
         <v>1.48</v>
       </c>
-      <c r="C481" t="inlineStr"/>
+      <c r="C481" t="n">
+        <v>43.35</v>
+      </c>
       <c r="D481" t="n">
         <v>58.5</v>
       </c>
@@ -15773,7 +15791,9 @@
       <c r="F481" t="n">
         <v>5.56</v>
       </c>
-      <c r="G481" t="inlineStr"/>
+      <c r="G481" t="n">
+        <v>70.04000000000001</v>
+      </c>
       <c r="H481" t="n">
         <v>64.88</v>
       </c>
@@ -15781,7 +15801,7 @@
         <v>2.18</v>
       </c>
       <c r="J481" t="n">
-        <v>24.21</v>
+        <v>35.67</v>
       </c>
     </row>
     <row r="482">
@@ -15791,7 +15811,9 @@
       <c r="B482" t="n">
         <v>1.48</v>
       </c>
-      <c r="C482" t="inlineStr"/>
+      <c r="C482" t="n">
+        <v>46.92</v>
+      </c>
       <c r="D482" t="n">
         <v>58.5</v>
       </c>
@@ -15801,7 +15823,9 @@
       <c r="F482" t="n">
         <v>5.75</v>
       </c>
-      <c r="G482" t="inlineStr"/>
+      <c r="G482" t="n">
+        <v>85.33</v>
+      </c>
       <c r="H482" t="n">
         <v>64.68000000000001</v>
       </c>
@@ -15809,7 +15833,7 @@
         <v>0.2</v>
       </c>
       <c r="J482" t="n">
-        <v>23.54</v>
+        <v>38.99</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-18 (sentiment: 47.42)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J483"/>
+  <dimension ref="A1:J484"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15890,7 +15890,7 @@
         <v>46.28</v>
       </c>
       <c r="E483" t="n">
-        <v>7.43</v>
+        <v>7.11</v>
       </c>
       <c r="F483" t="n">
         <v>4.96</v>
@@ -15902,10 +15902,42 @@
         <v>51.39</v>
       </c>
       <c r="I483" t="n">
-        <v>5.36</v>
+        <v>4.56</v>
       </c>
       <c r="J483" t="n">
-        <v>35.62</v>
+        <v>35.42</v>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" s="2" t="n">
+        <v>46283.66666666666</v>
+      </c>
+      <c r="B484" t="n">
+        <v>4.01</v>
+      </c>
+      <c r="C484" t="n">
+        <v>48.18</v>
+      </c>
+      <c r="D484" t="n">
+        <v>76.08</v>
+      </c>
+      <c r="E484" t="n">
+        <v>6.2</v>
+      </c>
+      <c r="F484" t="n">
+        <v>11.71</v>
+      </c>
+      <c r="G484" t="n">
+        <v>89.09</v>
+      </c>
+      <c r="H484" t="n">
+        <v>88.69</v>
+      </c>
+      <c r="I484" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J484" t="n">
+        <v>47.42</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-21 (sentiment: 50.60)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J484"/>
+  <dimension ref="A1:J485"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15922,7 +15922,7 @@
         <v>76.08</v>
       </c>
       <c r="E484" t="n">
-        <v>6.2</v>
+        <v>7.24</v>
       </c>
       <c r="F484" t="n">
         <v>11.71</v>
@@ -15934,10 +15934,34 @@
         <v>88.69</v>
       </c>
       <c r="I484" t="n">
-        <v>0.2</v>
+        <v>5.36</v>
       </c>
       <c r="J484" t="n">
-        <v>47.42</v>
+        <v>48.71</v>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" s="2" t="n">
+        <v>46286.66666666666</v>
+      </c>
+      <c r="B485" t="inlineStr"/>
+      <c r="C485" t="inlineStr"/>
+      <c r="D485" t="n">
+        <v>81.51000000000001</v>
+      </c>
+      <c r="E485" t="n">
+        <v>7.36</v>
+      </c>
+      <c r="F485" t="inlineStr"/>
+      <c r="G485" t="inlineStr"/>
+      <c r="H485" t="n">
+        <v>95.04000000000001</v>
+      </c>
+      <c r="I485" t="n">
+        <v>6.15</v>
+      </c>
+      <c r="J485" t="n">
+        <v>50.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-22 (sentiment: 24.21)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J485"/>
+  <dimension ref="A1:J486"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15950,7 +15950,7 @@
         <v>81.51000000000001</v>
       </c>
       <c r="E485" t="n">
-        <v>7.36</v>
+        <v>7.31</v>
       </c>
       <c r="F485" t="inlineStr"/>
       <c r="G485" t="inlineStr"/>
@@ -15958,10 +15958,34 @@
         <v>95.04000000000001</v>
       </c>
       <c r="I485" t="n">
-        <v>6.15</v>
+        <v>5.75</v>
       </c>
       <c r="J485" t="n">
-        <v>50.6</v>
+        <v>50.4</v>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" s="2" t="n">
+        <v>46287.66666666666</v>
+      </c>
+      <c r="B486" t="inlineStr"/>
+      <c r="C486" t="inlineStr"/>
+      <c r="D486" t="n">
+        <v>42.65</v>
+      </c>
+      <c r="E486" t="n">
+        <v>6.98</v>
+      </c>
+      <c r="F486" t="inlineStr"/>
+      <c r="G486" t="inlineStr"/>
+      <c r="H486" t="n">
+        <v>44.25</v>
+      </c>
+      <c r="I486" t="n">
+        <v>4.17</v>
+      </c>
+      <c r="J486" t="n">
+        <v>24.21</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-23 (sentiment: 35.32)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J486"/>
+  <dimension ref="A1:J487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15974,7 +15974,7 @@
         <v>42.65</v>
       </c>
       <c r="E486" t="n">
-        <v>6.98</v>
+        <v>7.79</v>
       </c>
       <c r="F486" t="inlineStr"/>
       <c r="G486" t="inlineStr"/>
@@ -15982,10 +15982,34 @@
         <v>44.25</v>
       </c>
       <c r="I486" t="n">
-        <v>4.17</v>
+        <v>6.94</v>
       </c>
       <c r="J486" t="n">
-        <v>24.21</v>
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" s="2" t="n">
+        <v>46288.66666666666</v>
+      </c>
+      <c r="B487" t="inlineStr"/>
+      <c r="C487" t="inlineStr"/>
+      <c r="D487" t="n">
+        <v>33.97</v>
+      </c>
+      <c r="E487" t="n">
+        <v>9.44</v>
+      </c>
+      <c r="F487" t="inlineStr"/>
+      <c r="G487" t="inlineStr"/>
+      <c r="H487" t="n">
+        <v>34.33</v>
+      </c>
+      <c r="I487" t="n">
+        <v>36.31</v>
+      </c>
+      <c r="J487" t="n">
+        <v>35.32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-24 (sentiment: 9.13)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J487"/>
+  <dimension ref="A1:J488"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -15998,7 +15998,7 @@
         <v>33.97</v>
       </c>
       <c r="E487" t="n">
-        <v>9.44</v>
+        <v>7.25</v>
       </c>
       <c r="F487" t="inlineStr"/>
       <c r="G487" t="inlineStr"/>
@@ -16006,10 +16006,34 @@
         <v>34.33</v>
       </c>
       <c r="I487" t="n">
-        <v>36.31</v>
+        <v>5.75</v>
       </c>
       <c r="J487" t="n">
-        <v>35.32</v>
+        <v>20.04</v>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" s="2" t="n">
+        <v>46289.66666666666</v>
+      </c>
+      <c r="B488" t="inlineStr"/>
+      <c r="C488" t="inlineStr"/>
+      <c r="D488" t="n">
+        <v>20.11</v>
+      </c>
+      <c r="E488" t="n">
+        <v>7.74</v>
+      </c>
+      <c r="F488" t="inlineStr"/>
+      <c r="G488" t="inlineStr"/>
+      <c r="H488" t="n">
+        <v>10.91</v>
+      </c>
+      <c r="I488" t="n">
+        <v>7.34</v>
+      </c>
+      <c r="J488" t="n">
+        <v>9.130000000000001</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-24 (sentiment: 20.93)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -16040,16 +16040,24 @@
       <c r="A488" s="2" t="n">
         <v>46289.66666666666</v>
       </c>
-      <c r="B488" t="inlineStr"/>
-      <c r="C488" t="inlineStr"/>
+      <c r="B488" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="C488" t="n">
+        <v>42.69</v>
+      </c>
       <c r="D488" t="n">
         <v>20.11</v>
       </c>
       <c r="E488" t="n">
         <v>7.74</v>
       </c>
-      <c r="F488" t="inlineStr"/>
-      <c r="G488" t="inlineStr"/>
+      <c r="F488" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="G488" t="n">
+        <v>64.88</v>
+      </c>
       <c r="H488" t="n">
         <v>10.91</v>
       </c>
@@ -16057,7 +16065,7 @@
         <v>7.34</v>
       </c>
       <c r="J488" t="n">
-        <v>9.130000000000001</v>
+        <v>20.93</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-09-30 (sentiment: 27.18)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J490"/>
+  <dimension ref="A1:J491"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16102,7 +16102,7 @@
         <v>62.32</v>
       </c>
       <c r="E490" t="n">
-        <v>7.72</v>
+        <v>6.97</v>
       </c>
       <c r="F490" t="inlineStr"/>
       <c r="G490" t="inlineStr"/>
@@ -16110,10 +16110,34 @@
         <v>71.23</v>
       </c>
       <c r="I490" t="n">
-        <v>7.74</v>
+        <v>4.56</v>
       </c>
       <c r="J490" t="n">
-        <v>39.48</v>
+        <v>37.9</v>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" s="2" t="n">
+        <v>46295.66666666666</v>
+      </c>
+      <c r="B491" t="inlineStr"/>
+      <c r="C491" t="inlineStr"/>
+      <c r="D491" t="n">
+        <v>46.06</v>
+      </c>
+      <c r="E491" t="n">
+        <v>6.82</v>
+      </c>
+      <c r="F491" t="inlineStr"/>
+      <c r="G491" t="inlineStr"/>
+      <c r="H491" t="n">
+        <v>50.6</v>
+      </c>
+      <c r="I491" t="n">
+        <v>3.77</v>
+      </c>
+      <c r="J491" t="n">
+        <v>27.18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-16 (sentiment: 34.13)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J497"/>
+  <dimension ref="A1:J498"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16334,7 +16334,7 @@
         <v>7.7</v>
       </c>
       <c r="E497" t="n">
-        <v>5.49</v>
+        <v>6.03</v>
       </c>
       <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr"/>
@@ -16348,6 +16348,30 @@
         <v>0.6</v>
       </c>
     </row>
+    <row r="498">
+      <c r="A498" s="2" t="n">
+        <v>46311.66666666666</v>
+      </c>
+      <c r="B498" t="inlineStr"/>
+      <c r="C498" t="inlineStr"/>
+      <c r="D498" t="n">
+        <v>59.2</v>
+      </c>
+      <c r="E498" t="n">
+        <v>6.33</v>
+      </c>
+      <c r="F498" t="inlineStr"/>
+      <c r="G498" t="inlineStr"/>
+      <c r="H498" t="n">
+        <v>66.47</v>
+      </c>
+      <c r="I498" t="n">
+        <v>1.79</v>
+      </c>
+      <c r="J498" t="n">
+        <v>34.13</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-20 (sentiment: 40.48)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J499"/>
+  <dimension ref="A1:J500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16394,7 +16394,7 @@
         <v>40.8</v>
       </c>
       <c r="E499" t="n">
-        <v>6.75</v>
+        <v>6.55</v>
       </c>
       <c r="F499" t="n">
         <v>1.39</v>
@@ -16406,10 +16406,34 @@
         <v>43.06</v>
       </c>
       <c r="I499" t="n">
-        <v>6.55</v>
+        <v>4.17</v>
       </c>
       <c r="J499" t="n">
-        <v>24.35</v>
+        <v>23.76</v>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" s="2" t="n">
+        <v>46315.66666666666</v>
+      </c>
+      <c r="B500" t="inlineStr"/>
+      <c r="C500" t="inlineStr"/>
+      <c r="D500" t="n">
+        <v>67.76000000000001</v>
+      </c>
+      <c r="E500" t="n">
+        <v>6.4</v>
+      </c>
+      <c r="F500" t="inlineStr"/>
+      <c r="G500" t="inlineStr"/>
+      <c r="H500" t="n">
+        <v>77.58</v>
+      </c>
+      <c r="I500" t="n">
+        <v>3.37</v>
+      </c>
+      <c r="J500" t="n">
+        <v>40.48</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data: auto-fetch & update sentiment data up to 2026-10-28 (sentiment: 43.25)
</commit_message>
<xml_diff>
--- a/docs/情绪指标_结果.xlsx
+++ b/docs/情绪指标_结果.xlsx
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J505"/>
+  <dimension ref="A1:J506"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -16586,7 +16586,7 @@
         <v>10.87</v>
       </c>
       <c r="E505" t="n">
-        <v>6.83</v>
+        <v>6.14</v>
       </c>
       <c r="F505" t="n">
         <v>2.59</v>
@@ -16598,10 +16598,34 @@
         <v>3.37</v>
       </c>
       <c r="I505" t="n">
-        <v>9.720000000000001</v>
+        <v>0.99</v>
       </c>
       <c r="J505" t="n">
-        <v>16.12</v>
+        <v>13.94</v>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" s="2" t="n">
+        <v>46323.66666666666</v>
+      </c>
+      <c r="B506" t="inlineStr"/>
+      <c r="C506" t="inlineStr"/>
+      <c r="D506" t="n">
+        <v>74.55</v>
+      </c>
+      <c r="E506" t="n">
+        <v>5.44</v>
+      </c>
+      <c r="F506" t="inlineStr"/>
+      <c r="G506" t="inlineStr"/>
+      <c r="H506" t="n">
+        <v>86.31</v>
+      </c>
+      <c r="I506" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="J506" t="n">
+        <v>43.25</v>
       </c>
     </row>
   </sheetData>

</xml_diff>